<commit_message>
river illustration, well 9, scenarios_short3.xlsx
the river channel is now included in the topology for coloration/visualization.

well 9 is now included in the scenarios files
</commit_message>
<xml_diff>
--- a/layered_groundwater_model/inputs/topology.xlsx
+++ b/layered_groundwater_model/inputs/topology.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krasows2\Documents\GitHub\isws-demonstration-models\layered_groundwater_model\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB84998B-3E83-44F5-9014-94026E8C76BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81F1CDBD-7198-4FED-A76F-D88E1FE9BF8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{43C37637-5F19-4EED-AAE4-F038FFA13CAD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{43C37637-5F19-4EED-AAE4-F038FFA13CAD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="15">
   <si>
     <t>id</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>inactive</t>
+  </si>
+  <si>
+    <t>river_channel</t>
   </si>
 </sst>
 </file>
@@ -455,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B430B04-988F-4B86-8623-4FDB30D2E834}">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
@@ -983,10 +986,10 @@
         <v>7</v>
       </c>
       <c r="B48">
-        <v>6.2</v>
+        <v>5.7</v>
       </c>
       <c r="C48">
-        <v>21.1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -994,10 +997,10 @@
         <v>7</v>
       </c>
       <c r="B49">
-        <v>11.3</v>
+        <v>6.2</v>
       </c>
       <c r="C49">
-        <v>21.4</v>
+        <v>21.1</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1005,10 +1008,10 @@
         <v>7</v>
       </c>
       <c r="B50">
-        <v>12.1</v>
+        <v>11.3</v>
       </c>
       <c r="C50">
-        <v>22.700000000000003</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1016,7 +1019,7 @@
         <v>7</v>
       </c>
       <c r="B51">
-        <v>19.3</v>
+        <v>12.1</v>
       </c>
       <c r="C51">
         <v>22.700000000000003</v>
@@ -1027,7 +1030,7 @@
         <v>7</v>
       </c>
       <c r="B52">
-        <v>29.5</v>
+        <v>19.3</v>
       </c>
       <c r="C52">
         <v>22.700000000000003</v>
@@ -1041,7 +1044,7 @@
         <v>29.5</v>
       </c>
       <c r="C53">
-        <v>21.9</v>
+        <v>22.700000000000003</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -1049,7 +1052,7 @@
         <v>7</v>
       </c>
       <c r="B54">
-        <v>34.5</v>
+        <v>29.5</v>
       </c>
       <c r="C54">
         <v>21.9</v>
@@ -1063,7 +1066,7 @@
         <v>34.5</v>
       </c>
       <c r="C55">
-        <v>22.700000000000003</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
@@ -1071,10 +1074,10 @@
         <v>7</v>
       </c>
       <c r="B56">
-        <v>51.2</v>
+        <v>34.5</v>
       </c>
       <c r="C56">
-        <v>24</v>
+        <v>22.700000000000003</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -1085,7 +1088,7 @@
         <v>51.2</v>
       </c>
       <c r="C57">
-        <v>22.6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -1093,10 +1096,10 @@
         <v>7</v>
       </c>
       <c r="B58">
-        <v>24.5</v>
+        <v>51.2</v>
       </c>
       <c r="C58">
-        <v>19.5</v>
+        <v>22.6</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -1104,106 +1107,106 @@
         <v>7</v>
       </c>
       <c r="B59">
-        <v>0</v>
+        <v>24.5</v>
       </c>
       <c r="C59">
-        <v>14.3</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B60">
-        <v>29.5</v>
+        <v>0</v>
       </c>
       <c r="C60">
-        <v>21.9</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B61">
-        <v>29.5</v>
+        <v>0</v>
       </c>
       <c r="C61">
-        <v>22.700000000000003</v>
+        <v>16.600000000000001</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B62">
-        <v>34.5</v>
+        <v>0</v>
       </c>
       <c r="C62">
-        <v>22.700000000000003</v>
+        <v>20</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B63">
-        <v>34.5</v>
+        <v>5.7</v>
       </c>
       <c r="C63">
-        <v>21.9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B64">
-        <v>29.5</v>
+        <v>4.2</v>
       </c>
       <c r="C64">
-        <v>21.9</v>
+        <v>16.600000000000001</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B65">
-        <v>12.1</v>
+        <v>0</v>
       </c>
       <c r="C65">
-        <v>22.700000000000003</v>
+        <v>16.600000000000001</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B66">
-        <v>12.5</v>
+        <v>29.5</v>
       </c>
       <c r="C66">
-        <v>23.5</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B67">
-        <v>19.3</v>
+        <v>29.5</v>
       </c>
       <c r="C67">
-        <v>23.5</v>
+        <v>22.700000000000003</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B68">
-        <v>19.3</v>
+        <v>34.5</v>
       </c>
       <c r="C68">
         <v>22.700000000000003</v>
@@ -1211,79 +1214,79 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B69">
-        <v>12.1</v>
+        <v>34.5</v>
       </c>
       <c r="C69">
-        <v>22.700000000000003</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B70">
-        <v>12.5</v>
+        <v>29.5</v>
       </c>
       <c r="C70">
-        <v>23.5</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B71">
-        <v>13.6</v>
+        <v>12.1</v>
       </c>
       <c r="C71">
-        <v>25.6</v>
+        <v>22.700000000000003</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B72">
-        <v>21.4</v>
+        <v>12.5</v>
       </c>
       <c r="C72">
-        <v>26.6</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B73">
-        <v>28.5</v>
+        <v>19.3</v>
       </c>
       <c r="C73">
-        <v>27.3</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B74">
-        <v>51.2</v>
+        <v>19.3</v>
       </c>
       <c r="C74">
-        <v>28.1</v>
+        <v>22.700000000000003</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B75">
-        <v>51.2</v>
+        <v>12.1</v>
       </c>
       <c r="C75">
-        <v>24</v>
+        <v>22.700000000000003</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
@@ -1291,10 +1294,10 @@
         <v>10</v>
       </c>
       <c r="B76">
-        <v>34.5</v>
+        <v>12.5</v>
       </c>
       <c r="C76">
-        <v>22.700000000000003</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
@@ -1302,10 +1305,10 @@
         <v>10</v>
       </c>
       <c r="B77">
-        <v>29.5</v>
+        <v>13.6</v>
       </c>
       <c r="C77">
-        <v>22.700000000000003</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
@@ -1313,10 +1316,10 @@
         <v>10</v>
       </c>
       <c r="B78">
-        <v>19.3</v>
+        <v>21.4</v>
       </c>
       <c r="C78">
-        <v>22.700000000000003</v>
+        <v>26.6</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
@@ -1324,10 +1327,10 @@
         <v>10</v>
       </c>
       <c r="B79">
-        <v>19.3</v>
+        <v>28.5</v>
       </c>
       <c r="C79">
-        <v>23.5</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
@@ -1335,76 +1338,76 @@
         <v>10</v>
       </c>
       <c r="B80">
-        <v>12.5</v>
+        <v>51.2</v>
       </c>
       <c r="C80">
-        <v>23.5</v>
+        <v>28.1</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B81">
-        <v>0</v>
+        <v>51.2</v>
       </c>
       <c r="C81">
-        <v>16.600000000000001</v>
+        <v>24</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B82">
-        <v>0</v>
+        <v>34.5</v>
       </c>
       <c r="C82">
-        <v>29.8</v>
+        <v>22.700000000000003</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B83">
-        <v>51.2</v>
+        <v>29.5</v>
       </c>
       <c r="C83">
-        <v>29.8</v>
+        <v>22.700000000000003</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B84">
-        <v>51.2</v>
+        <v>19.3</v>
       </c>
       <c r="C84">
-        <v>28.1</v>
+        <v>22.700000000000003</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B85">
-        <v>28.5</v>
+        <v>19.3</v>
       </c>
       <c r="C85">
-        <v>27.3</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B86">
-        <v>21.4</v>
+        <v>12.5</v>
       </c>
       <c r="C86">
-        <v>26.6</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
@@ -1412,10 +1415,10 @@
         <v>13</v>
       </c>
       <c r="B87">
-        <v>13.6</v>
+        <v>0</v>
       </c>
       <c r="C87">
-        <v>25.6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
@@ -1423,10 +1426,10 @@
         <v>13</v>
       </c>
       <c r="B88">
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="C88">
-        <v>23.5</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
@@ -1434,10 +1437,10 @@
         <v>13</v>
       </c>
       <c r="B89">
-        <v>12.1</v>
+        <v>51.2</v>
       </c>
       <c r="C89">
-        <v>22.700000000000003</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
@@ -1445,10 +1448,10 @@
         <v>13</v>
       </c>
       <c r="B90">
-        <v>11.3</v>
+        <v>51.2</v>
       </c>
       <c r="C90">
-        <v>21.4</v>
+        <v>28.1</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
@@ -1456,10 +1459,10 @@
         <v>13</v>
       </c>
       <c r="B91">
-        <v>6.2</v>
+        <v>28.5</v>
       </c>
       <c r="C91">
-        <v>21.1</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
@@ -1467,10 +1470,10 @@
         <v>13</v>
       </c>
       <c r="B92">
-        <v>4.2</v>
+        <v>21.4</v>
       </c>
       <c r="C92">
-        <v>16.600000000000001</v>
+        <v>26.6</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
@@ -1478,10 +1481,76 @@
         <v>13</v>
       </c>
       <c r="B93">
-        <v>0</v>
+        <v>13.6</v>
       </c>
       <c r="C93">
-        <v>16.600000000000001</v>
+        <v>25.6</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>13</v>
+      </c>
+      <c r="B94">
+        <v>12.5</v>
+      </c>
+      <c r="C94">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>13</v>
+      </c>
+      <c r="B95">
+        <v>12.1</v>
+      </c>
+      <c r="C95">
+        <v>22.700000000000003</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>13</v>
+      </c>
+      <c r="B96">
+        <v>11.3</v>
+      </c>
+      <c r="C96">
+        <v>21.4</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>13</v>
+      </c>
+      <c r="B97">
+        <v>6.2</v>
+      </c>
+      <c r="C97">
+        <v>21.1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>13</v>
+      </c>
+      <c r="B98">
+        <v>5.7</v>
+      </c>
+      <c r="C98">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>13</v>
+      </c>
+      <c r="B99">
+        <v>0</v>
+      </c>
+      <c r="C99">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>